<commit_message>
Sample data: label duplicate Function IDs 旧仕様 / 新仕様 + add gap case
The old sample already had two adjacent duplicates (SEARCH01, PAY001)
but the names were neutral, so the loader's "last occurrence wins"
behavior wasn't visually obvious. Renamed every duplicate to
"... (旧仕様 — 上書き対象)" / "... (新仕様 — 採用される)" so the
intent is clear when you open function_master.xlsx and compare with
the dashboard — only the 新仕様 rows should appear downstream.

Also added a non-adjacent USER010 duplicate (the original sits in the
USER block, the duplicate sits between EXP001 and IMP001) to exercise
the "duplicates with rows in between" path, not just the adjacent
case.

Result: 21 source rows → 18 unique 機能IDs after dedup.

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample_data/function_master.xlsx
+++ b/sample_data/function_master.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,11 +465,6 @@
           <t>Notes</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>機能概要</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -505,11 +500,6 @@
           <t>User Login</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>メールアドレスとパスワードでログイン認証を行う。失敗回数のロックアウト、SAML/OIDC連携、二要素認証(TOTP)に対応。</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -545,11 +535,6 @@
           <t>User Registration</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>新規ユーザー登録フォーム。メール検証トークンの送付・有効化、利用規約同意の記録、reCAPTCHA連携を含む。</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -585,11 +570,6 @@
           <t>Password Reset</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>パスワード忘却時の再設定フロー。本人確認メール経由のワンタイムリンクと、24時間の有効期限管理を行う。</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -622,12 +602,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Profile Edit</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>ユーザー本人によるプロフィール編集。表示名、アイコン、通知設定、タイムゾーンを更新できる。</t>
+          <t>Profile Edit (旧仕様 — 上書き対象)</t>
         </is>
       </c>
     </row>
@@ -665,11 +640,6 @@
           <t>Profile Edit (Admin)</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>管理者によるプロフィール編集。所属、権限ロール、停止/復活フラグなど一般ユーザーには触れない項目を含む。</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
@@ -709,12 +679,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Search (Basic)</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>全文検索の基本機能。商品名・説明文に対するキーワードマッチと、件数ベースのページング表示を提供する。</t>
+          <t>Search (Basic 旧仕様 — 上書き対象)</t>
         </is>
       </c>
     </row>
@@ -749,12 +714,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Search (Advanced)</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>高度な検索フィルタ。価格帯・在庫状況・カテゴリ・タグの複合条件と、ファセットUIによる絞り込みに対応。</t>
+          <t>Search (Advanced 新仕様 — 採用される)</t>
         </is>
       </c>
     </row>
@@ -792,11 +752,6 @@
           <t>Cart Add</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>カートへの商品追加。在庫引当はせず、購入確定時に再検証する楽観方式。SKU単位で数量管理する。</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -832,11 +787,6 @@
           <t>Cart Remove</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>カートからの商品削除と数量変更。削除取り消しのスナックバーUIをWebフロントで提供する。</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -872,11 +822,6 @@
           <t>Checkout</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>チェックアウトフロー。配送先・支払い方法・クーポン適用・合計金額の確認を経て注文を確定する。</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="B13" t="inlineStr">
@@ -916,12 +861,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Payment - Credit Card</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>クレジットカード決済。3DS2.0認証、決済代行APIとの連携、決済失敗時のリトライポリシーを持つ。</t>
+          <t>Payment - Credit Card (旧仕様 — 上書き対象)</t>
         </is>
       </c>
     </row>
@@ -956,12 +896,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Payment - Bank Transfer</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>銀行振込決済。仮想口座番号の自動採番、入金照合バッチ、未入金リマインダ送信を含む。</t>
+          <t>Payment - Bank Transfer (新仕様 — 採用される)</t>
         </is>
       </c>
     </row>
@@ -999,11 +934,6 @@
           <t>Order History</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>ユーザー自身の過去注文一覧。直近24ヶ月分を表示し、領収書PDFダウンロードに対応する。</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1039,11 +969,6 @@
           <t>Notification - Email</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>メール通知の送信機能。テンプレート展開、配信ステータス追跡、バウンス処理を行う。</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1079,11 +1004,6 @@
           <t>Notification - Push</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>プッシュ通知。FCM/APNs両対応、ユーザーごとの通知許可設定とサイレント時間帯の制御を行う。</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1119,11 +1039,6 @@
           <t>Settings Sync</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>アプリ設定の端末間同期。差分マージとコンフリクト解決(最終更新優先)を実装する。</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1159,11 +1074,6 @@
           <t>Data Export</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>データエクスポート機能。CSV/Excel形式での出力と、大量データ時の非同期ジョブ化に対応。</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1191,103 +1101,123 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
+          <t>USER010</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Profile Edit (新仕様 — 採用される)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Worker</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>bob</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
           <t>IMP001</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>Data Import</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>データインポート機能。CSVフォーマットの検証、エラー行のレポート、ロールバック処理を含む。</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Admin</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Worker</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>bob</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>carol</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>AUDIT01</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>Audit Log</t>
         </is>
       </c>
-      <c r="H22" s="2" t="n"/>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>監査ログ。重要操作の不可変ログ記録と、検索・フィルタ・CSV出力UIを提供する。</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>20</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>User</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>API</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>carol</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
+      <c r="H23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>alice</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Deprecated</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
         <is>
           <t>ADM001</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>Admin Dashboard</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>管理者向けダッシュボード。利用状況・障害アラート・リクエスト数の主要KPIを集約表示する。</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" t="inlineStr">
+    </row>
+    <row r="27">
+      <c r="B27" t="inlineStr">
         <is>
           <t>Total</t>
         </is>

</xml_diff>